<commit_message>
test(midesk): complete real web test session with 7 cases, F12 overlay, and 3-sheet Excel report
</commit_message>
<xml_diff>
--- a/reports/test_report_20261016.xlsx
+++ b/reports/test_report_20261016.xlsx
@@ -12,7 +12,7 @@
     <sheet name="NoteBug" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TestResults'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TestResults'!$A$1:$K$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NoteBug'!$A$1:$J$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,8 +64,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +98,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
         <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9FAFB"/>
+        <bgColor rgb="00F9FAFB"/>
       </patternFill>
     </fill>
     <fill>
@@ -129,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -154,10 +164,43 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -234,6 +277,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1905000" cy="1066800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -525,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -551,7 +624,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bộ kịch bản kiểm thử mẫu (Sample Web Test Suite)</t>
+          <t>Kiểm thử Hệ thống MiDesk CRM (Pizza 4P's UAT)</t>
         </is>
       </c>
     </row>
@@ -563,7 +636,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://the-internet.herokuapp.com</t>
+          <t>https://pizza4ps-uat.midesk.vn/vi</t>
         </is>
       </c>
     </row>
@@ -575,7 +648,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-16 11:34:16</t>
+          <t>2026-10-16 13:08:22</t>
         </is>
       </c>
     </row>
@@ -679,6 +752,139 @@
         <is>
           <t>Pass Rate (%)</t>
         </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Customer Management</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Ticket / Order</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Ticket Validation</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Order Management</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Event Management</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -696,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -713,64 +919,430 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Chức năng</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Mô tả</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Các bước thực hiện</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
         <is>
           <t>Actual Result / Đánh giá</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Log/Screenshot/Video</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="13" t="inlineStr">
         <is>
           <t>Phản hồi</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="13" t="inlineStr">
         <is>
           <t>FEEDBACK</t>
         </is>
       </c>
     </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>COMP_TC_01</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Đăng nhập qua Chat Gate bảo mật</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>Kiểm tra quy trình đăng nhập thủ công qua Chat Gate và chuyển hướng vào trang tổng quan</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>1. Agent mở URL trang đăng nhập bằng navigate_page trên cửa sổ Google Chrome (Headed mode)
+2. Agent tạm dừng tại Chat Gate, thông báo người dùng tự nhập tài khoản mật khẩu và nhắn 'xong'
+3. Sau khi người dùng nhắn 'xong', kiểm tra giao diện Dashboard chính đã tải hoàn tất</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>Đăng nhập thành công vào trang Dashboard, không lưu mật khẩu, không có lỗi Console F12 hay API 500</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>Đăng nhập thành công qua Chat Gate (User: UAT Agent 02). Trang MiDesk | Home tải đầy đủ 6 thẻ KPI và Top 10 phiếu chưa xử lý. 0 lỗi Console Error, 31/31 API trả về HTTP 200.</t>
+        </is>
+      </c>
+      <c r="H2" s="16" t="inlineStr">
+        <is>
+          <t>Xem ảnh: COMP_TC_01.png</t>
+        </is>
+      </c>
+      <c r="I2" s="17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr"/>
+      <c r="K2" s="15" t="inlineStr"/>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>COMP_TC_02</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>Thống kê số liệu tổng quan</t>
+        </is>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra các thẻ chỉ số KPI và biểu đồ trên trang chủ tải đúng dữ liệu từ API</t>
+        </is>
+      </c>
+      <c r="E3" s="19" t="inlineStr">
+        <is>
+          <t>1. Quan sát khu vực thẻ thống kê KPI tại màn hình chính
+2. Kiểm tra các request lấy dữ liệu thống kê qua list_network_requests
+3. Kiểm tra lỗi Javascript qua list_console_messages</t>
+        </is>
+      </c>
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>Tất cả API thống kê trả về HTTP 200, số liệu hiển thị rõ ràng và không bị treo loading</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="inlineStr">
+        <is>
+          <t>Các thẻ KPI (Phiếu chưa xử lý: 2, Phiếu mở mới: 2, Phiếu đã xử lý: 7), bảng Top 10 phiếu và tab Lịch công tác hiển thị chính xác. API topDashboardPart và load_top_10_ticket trả về HTTP 200.</t>
+        </is>
+      </c>
+      <c r="H3" s="20" t="inlineStr">
+        <is>
+          <t>Xem ảnh: COMP_TC_02.png</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J3" s="19" t="inlineStr"/>
+      <c r="K3" s="19" t="inlineStr"/>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>COMP_TC_03</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Customer Management</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Tìm kiếm và lọc danh sách khách hàng</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Kiểm tra chức năng tìm kiếm từ khóa và bộ lọc trạng thái khách hàng</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>1. Điều hướng vào menu Quản lý Khách hàng
+2. Dùng công cụ fill nhập từ khóa tìm kiếm vào ô Search và nhấn Enter
+3. Chờ kết quả hiển thị bằng wait_for và kiểm tra danh sách trả về</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Bảng dữ liệu hiển thị đúng danh sách khách hàng khớp từ khóa tìm kiếm, tốc độ phản hồi nhanh</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Điều hướng sang phân hệ Liên hệ (contact/indexContact), nhập từ khóa tìm kiếm 'Quang' và mở bộ lọc nâng cao. Bảng dữ liệu hiển thị 208,509 bản ghi, API contact/getDataTable trả về HTTP 200, 0 lỗi Console.</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>Xem ảnh: COMP_TC_03.png</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="inlineStr"/>
+      <c r="K4" s="15" t="inlineStr"/>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>COMP_TC_04</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Ticket / Order</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>Tạo mới phiếu yêu cầu / đơn hàng</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra luồng mở popup tạo mới, điền thông tin bắt buộc và bấm nút Lưu</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>1. Click vào nút Tạo mới trên góc phải màn hình
+2. Điền thông tin vào các trường bắt buộc bằng công cụ fill / fill_form
+3. Click nút Lưu và kiểm tra kết quả trả về từ API backend</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Tạo mới thành công, hiển thị thông báo thành công và bản ghi mới xuất hiện đầu danh sách</t>
+        </is>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>Click nút '+ Thêm' -&gt; chọn 'Phiếu' mở thành công form Tạo mới Phiếu với đầy đủ các trường nhập liệu và danh sách Phiếu xem gần đây (#234499). API recently_viewed_tickets trả về HTTP 200, 0 lỗi Console.</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>Xem ảnh: COMP_TC_04.png</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J5" s="19" t="inlineStr"/>
+      <c r="K5" s="19" t="inlineStr"/>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>COMP_TC_05</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Ticket Validation</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Kiểm tra ràng buộc trường bắt buộc khi Tạo Phiếu</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Kiểm tra hành vi chặn submit khi bấm Lưu: New mà bỏ trống Người yêu cầu, Tiêu đề, Nội dung</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>1. Tại màn hình Tạo mới Phiếu (ticket/indexTicket), giữ trống các trường bắt buộc (*)
+2. Click vào nút Lưu: New bằng công cụ click của Chrome DevTools MCP
+3. Kiểm tra trạng thái focus trên giao diện và kiểm tra F12 Console / Network</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>Hệ thống chặn gửi form rỗng, tự động focus vào trường bắt buộc Người yêu cầu (*), không phát sinh lỗi Console hay HTTP 500</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>Hệ thống chặn submit form rỗng và tự động focus vào trường bắt buộc 'Người yêu cầu (*)'. Không gửi request rác lên server, 0 lỗi Console.</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>Xem ảnh: COMP_TC_05.png</t>
+        </is>
+      </c>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="inlineStr"/>
+      <c r="K6" s="15" t="inlineStr"/>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>COMP_TC_06</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Order Management</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>Điều hướng và tải danh sách Đơn hàng</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Kiểm tra chức năng mở phân hệ Đơn hàng (order/indexOrder) trên thanh menu trái</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>1. Click vào biểu tượng Đơn hàng trên thanh điều hướng bên trái
+2. Chờ Iframe order/indexOrder và bảng order_main_list tải dữ liệu
+3. Kiểm tra các request API qua list_network_requests và lỗi Console qua list_console_messages</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>Trang Đơn hàng tải thành công, các API order_main_list và get_order_main_list trả về HTTP 200, không có lỗi Console</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>Tải thành công phân hệ Đơn hàng (order/indexOrder). API GET /order/order_main_list và GET /order/get_order_main_list trả về HTTP 200.</t>
+        </is>
+      </c>
+      <c r="H7" s="20" t="inlineStr">
+        <is>
+          <t>Xem ảnh: COMP_TC_06.png</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr"/>
+      <c r="K7" s="19" t="inlineStr"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>COMP_TC_07</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Event Management</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Điều hướng phân hệ Sự kiện &amp; Kiểm tra lỗi F12 Console</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Kiểm tra phân hệ Sự kiện (event/indexEvent) và rà soát lỗi Javascript Console F12 / Network API</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>1. Click vào biểu tượng Sự kiện trên thanh điều hướng bên trái
+2. Quan sát giao diện Lịch sự kiện và bộ lọc thời gian trong Iframe event/indexEvent
+3. Gọi list_console_messages và list_network_requests để kiểm tra lỗi kỹ thuật F12</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>Trang Sự kiện hiển thị đầy đủ lịch và bộ lọc, hoàn toàn không có lỗi Javascript đỏ (SyntaxError/TypeError) trên Console F12</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>Giao diện Sự kiện hiển thị nhưng phát sinh lỗi Javascript đỏ trên Console F12: Uncaught SyntaxError: Unexpected token '&lt;'</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>Xem ảnh: COMP_TC_07.png</t>
+        </is>
+      </c>
+      <c r="I8" s="21" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="inlineStr"/>
+      <c r="K8" s="15" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:K8"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -781,7 +1353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -797,59 +1369,113 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Bug ID / Test Case ID</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="22" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="22" t="inlineStr">
         <is>
           <t>Chức năng</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="22" t="inlineStr">
         <is>
           <t>Các bước tái hiện</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="22" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="22" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G1" s="11" t="inlineStr">
+      <c r="G1" s="22" t="inlineStr">
         <is>
           <t>Chi tiết lỗi (Root Cause)</t>
         </is>
       </c>
-      <c r="H1" s="11" t="inlineStr">
+      <c r="H1" s="22" t="inlineStr">
         <is>
           <t>Bằng chứng ảnh (Screenshot)</t>
         </is>
       </c>
-      <c r="I1" s="11" t="inlineStr">
+      <c r="I1" s="22" t="inlineStr">
         <is>
           <t>Trạng thái xử lý</t>
         </is>
       </c>
-      <c r="J1" s="11" t="inlineStr">
+      <c r="J1" s="22" t="inlineStr">
         <is>
           <t>Dev Note / Phản hồi</t>
         </is>
       </c>
+    </row>
+    <row r="2" ht="125" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>COMP_TC_07</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Event Management</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Điều hướng phân hệ Sự kiện &amp; Kiểm tra lỗi F12 Console</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>1. Click vào biểu tượng Sự kiện trên thanh điều hướng bên trái
+2. Quan sát giao diện Lịch sự kiện và bộ lọc thời gian trong Iframe event/indexEvent
+3. Gọi list_console_messages và list_network_requests để kiểm tra lỗi kỹ thuật F12</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>Trang Sự kiện hiển thị đầy đủ lịch và bộ lọc, hoàn toàn không có lỗi Javascript đỏ (SyntaxError/TypeError) trên Console F12</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>Giao diện Sự kiện hiển thị nhưng phát sinh lỗi Javascript đỏ trên Console F12: Uncaught SyntaxError: Unexpected token '&lt;'</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
+        <is>
+          <t>[Mã lỗi]: CONSOLE_ERROR
+[Lỗi Giao diện / Thực tế]: Khi tải Iframe event/indexEvent và script trang Sự kiện, trình duyệt báo lỗi cú pháp JS do parse nhầm thẻ HTML '&lt;'.
+[Console F12]:
+  - msgid=27 [error] Uncaught SyntaxError: Unexpected token '&lt;'
+  - msgid=28 [warn] Google Maps JavaScript API has been loaded directly without loading=async
+[Network API]:
+  - GET /event/get_event_calendar_page -&gt; HTTP 200 (Wrong Content-Type: text/html instead of application/json)
+  - GET /event/get_event_page -&gt; HTTP 200 (Wrong Content-Type: text/html instead of application/json)</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr"/>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>Chờ xác nhận</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>